<commit_message>
fix(assets): Download and verify accurately matched 1-letter word pixel assets from AetherForgeAI API
</commit_message>
<xml_diff>
--- a/word_card_master_300.xlsx
+++ b/word_card_master_300.xlsx
@@ -453,17 +453,6 @@
           <t>한글 활자 디펜스 마스터 데이터북 (15종 핵심 자모 조합 체계)</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
-      <c r="G1" t="inlineStr"/>
-      <c r="H1" t="inlineStr"/>
-      <c r="I1" t="inlineStr"/>
-      <c r="J1" t="inlineStr"/>
-      <c r="K1" t="inlineStr"/>
-      <c r="L1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -579,7 +568,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>res://assets/05_회복_치유/persimmon_감/persimmon_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_감_persimmon_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -635,7 +624,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_장비/armor_갑/armor_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_갑_armor_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -691,7 +680,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/dog_개/dog_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_개_dog_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -747,7 +736,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>res://assets/map_ui/ui_gold_pixel_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_검_sword_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -803,7 +792,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/pickaxe_곡/pickaxe_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_곡_pickaxe_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -859,7 +848,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/mace_골/mace_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_골_mace_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -915,7 +904,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bear_곰/bear_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_곰_bear_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -971,7 +960,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>res://assets/map_ui/ui_gold_pixel_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_궁_bow_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1016,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/fist_권/fist_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_권_fist_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1072,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/trident_극/trident_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_극_spear_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1128,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>res://assets/06_버프_유틸/ki_기/ki_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_기_aura_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1184,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/blade_날/blade_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_날_blade_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1240,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/scythe_낫/scythe_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_낫_scythe_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1296,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>res://assets/map_ui/ui_gold_pixel_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_낮_sun_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1352,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/cold_냉/cold_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_냉_cold_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1408,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/thunder_뇌/thunder_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_뇌_lightning_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1464,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>res://assets/map_ui/ui_gold_pixel_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_눈_snow_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1520,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/moon_달/moon_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_달_moon_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1576,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>res://assets/map_ui/ui_gold_pixel_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_도_katana_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1632,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/poison_독/poison_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_독_poison_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1688,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>res://assets/map_ui/ui_gold_pixel_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_돌_stone_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1744,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>res://assets/05_회복_치유/yam_마/yam_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_마_herb_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1800,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_장비/barrier_막/barrier_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_막_barrier_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1856,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/horse_말/horse_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_말_horse_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1912,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>res://assets/06_버프_유틸/net_망/net_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_망_net_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -1979,7 +1968,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/spike_못/spike_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_못_spike_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2024,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>res://assets/05_회복_치유/radish_무/radish_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_무_radish_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2080,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>res://assets/05_회복_치유/jelly_묵/jelly_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_묵_jelly_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2136,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_장비/gate_문/gate_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_문_gate_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2203,7 +2192,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/water_물/water_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_물_water_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2248,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_장비/shield_방/shield_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_방_shield_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2304,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/snake_뱀/snake_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_뱀_snake_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2360,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bee_벌/bee_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_벌_bee_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2416,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/staff_봉/staff_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_봉_staff_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2472,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>res://assets/06_버프_유틸/drum_북/drum_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_북_drum_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2528,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/fire_불/fire_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_불_fire_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2584,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>res://assets/map_ui/ui_gold_pixel_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_비_rain_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2640,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>res://assets/03_원소_마법/ice_빙/ice_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_빙_ice_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2696,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/wind_slash_삭/wind_slash_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_삭_slash_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2752,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_장비/mountain_산/mountain_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_산_mountain_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2819,7 +2808,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bird_새/bird_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_새_bird_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2864,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>res://assets/05_회복_치유/spring_샘/spring_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_샘_spring_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2920,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>res://assets/05_회복_치유/life_생/life_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_생_life_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -2987,7 +2976,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_장비/castle_성/castle_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_성_castle_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -3043,7 +3032,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/bull_소/bull_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_소_bull_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -3099,7 +3088,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/iron_쇠/iron_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_쇠_iron_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3144,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>res://assets/05_회복_치유/breath_숨/breath_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_숨_breath_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3200,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_장비/guard_완/guard_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_완_guard_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3256,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_장비/orbit_위/orbit_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_위_orbit_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3312,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>res://assets/02_방어_장비/patience_인/patience_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_인_patience_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3368,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>res://assets/01_무기_공격/strike_일/strike_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_일_strike_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3424,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>res://assets/04_생물_소환/rat_쥐/rat_1_32px_pastel.png</t>
+          <t>res://assets/words_1letter/word_1_쥐_rat_32px_pastel.png</t>
         </is>
       </c>
     </row>
@@ -10464,8 +10453,6 @@
           <t>시작덱 기본 구성 (불 타워)</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -10508,7 +10495,6 @@
           <t>ㅜ</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -10519,7 +10505,6 @@
           <t>ㄹ</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10547,9 +10532,6 @@
           <t>15종 핵심 자모 타일 풀 (제외: ㅑㅕㅛㅠ, ㅋㅌㅊㅍㅎ)</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">

</xml_diff>